<commit_message>
Bangladesh + Thailand gas pulls: branch run
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/thailand_gas.xlsx
+++ b/output/Data and Chart Outputs/thailand_gas.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Production by field" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart - Demand" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supply" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Units" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Chart" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chart - Production by field" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Chart - Demand" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Supply" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Demand" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,8 +23,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="165" formatCode="mmm/yy"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="mmm/yy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -64,13 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -148,13 +147,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -179,10 +178,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -207,10 +206,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -235,10 +234,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -271,8 +270,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-2700000" vert="horz"/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -298,8 +297,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -316,7 +315,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -330,7 +329,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:ln>
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -339,13 +338,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -370,10 +369,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -398,10 +397,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -426,10 +425,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -454,10 +453,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -482,10 +481,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="E87BA4"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -510,10 +509,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="008300"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -538,10 +537,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="4A3AA7"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -574,8 +573,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-2700000" vert="horz"/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -601,8 +600,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -619,7 +618,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -633,7 +632,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:ln>
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -642,13 +641,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -673,10 +672,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -701,10 +700,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="EB6834"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -729,10 +728,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="1BAF7A"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -757,10 +756,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="EDA100"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -793,8 +792,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-2700000" vert="horz"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-2700000" vert="horz"/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -820,8 +819,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -838,7 +837,7 @@
         <crossAx val="10"/>
       </valAx>
       <spPr>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -852,7 +851,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:ln>
       <a:noFill/>
       <a:prstDash val="solid"/>
     </a:ln>
@@ -861,7 +860,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>5</col>
@@ -876,9 +875,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -888,7 +887,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -903,9 +902,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -915,7 +914,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -930,9 +929,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1271,6 +1270,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -1292,6 +1292,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
@@ -1346,7 +1347,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="3" t="n">
         <v>42005</v>
       </c>
       <c r="B2" t="n">
@@ -1360,7 +1361,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="3" t="n">
         <v>42036</v>
       </c>
       <c r="B3" t="n">
@@ -1374,7 +1375,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="3" t="n">
         <v>42064</v>
       </c>
       <c r="B4" t="n">
@@ -1388,7 +1389,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="3" t="n">
         <v>42095</v>
       </c>
       <c r="B5" t="n">
@@ -1402,7 +1403,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="3" t="n">
         <v>42125</v>
       </c>
       <c r="B6" t="n">
@@ -1416,7 +1417,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="3" t="n">
         <v>42156</v>
       </c>
       <c r="B7" t="n">
@@ -1430,7 +1431,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="3" t="n">
         <v>42186</v>
       </c>
       <c r="B8" t="n">
@@ -1444,7 +1445,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="3" t="n">
         <v>42217</v>
       </c>
       <c r="B9" t="n">
@@ -1458,7 +1459,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="3" t="n">
         <v>42248</v>
       </c>
       <c r="B10" t="n">
@@ -1472,7 +1473,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="3" t="n">
         <v>42278</v>
       </c>
       <c r="B11" t="n">
@@ -1486,7 +1487,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="3" t="n">
         <v>42309</v>
       </c>
       <c r="B12" t="n">
@@ -1500,7 +1501,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="3" t="n">
         <v>42339</v>
       </c>
       <c r="B13" t="n">
@@ -1514,7 +1515,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="3" t="n">
         <v>42370</v>
       </c>
       <c r="B14" t="n">
@@ -1528,7 +1529,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="3" t="n">
         <v>42401</v>
       </c>
       <c r="B15" t="n">
@@ -1542,7 +1543,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="3" t="n">
         <v>42430</v>
       </c>
       <c r="B16" t="n">
@@ -1556,7 +1557,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="3" t="n">
         <v>42461</v>
       </c>
       <c r="B17" t="n">
@@ -1570,7 +1571,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="3" t="n">
         <v>42491</v>
       </c>
       <c r="B18" t="n">
@@ -1584,7 +1585,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="3" t="n">
         <v>42522</v>
       </c>
       <c r="B19" t="n">
@@ -1598,7 +1599,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="3" t="n">
         <v>42552</v>
       </c>
       <c r="B20" t="n">
@@ -1612,7 +1613,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="3" t="n">
         <v>42583</v>
       </c>
       <c r="B21" t="n">
@@ -1626,7 +1627,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="3" t="n">
         <v>42614</v>
       </c>
       <c r="B22" t="n">
@@ -1640,7 +1641,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="3" t="n">
         <v>42644</v>
       </c>
       <c r="B23" t="n">
@@ -1654,7 +1655,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="3" t="n">
         <v>42675</v>
       </c>
       <c r="B24" t="n">
@@ -1668,7 +1669,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="3" t="n">
         <v>42705</v>
       </c>
       <c r="B25" t="n">
@@ -1682,7 +1683,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="3" t="n">
         <v>42736</v>
       </c>
       <c r="B26" t="n">
@@ -1696,7 +1697,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="3" t="n">
         <v>42767</v>
       </c>
       <c r="B27" t="n">
@@ -1710,7 +1711,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="3" t="n">
         <v>42795</v>
       </c>
       <c r="B28" t="n">
@@ -1724,7 +1725,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="3" t="n">
         <v>42826</v>
       </c>
       <c r="B29" t="n">
@@ -1738,7 +1739,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="3" t="n">
         <v>42856</v>
       </c>
       <c r="B30" t="n">
@@ -1752,7 +1753,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="3" t="n">
         <v>42887</v>
       </c>
       <c r="B31" t="n">
@@ -1766,7 +1767,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="3" t="n">
         <v>42917</v>
       </c>
       <c r="B32" t="n">
@@ -1780,7 +1781,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="3" t="n">
         <v>42948</v>
       </c>
       <c r="B33" t="n">
@@ -1794,7 +1795,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n">
+      <c r="A34" s="3" t="n">
         <v>42979</v>
       </c>
       <c r="B34" t="n">
@@ -1808,7 +1809,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="3" t="n">
         <v>43009</v>
       </c>
       <c r="B35" t="n">
@@ -1822,7 +1823,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="3" t="n">
         <v>43040</v>
       </c>
       <c r="B36" t="n">
@@ -1836,7 +1837,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="3" t="n">
         <v>43070</v>
       </c>
       <c r="B37" t="n">
@@ -1850,7 +1851,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n">
+      <c r="A38" s="3" t="n">
         <v>43101</v>
       </c>
       <c r="B38" t="n">
@@ -1864,7 +1865,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="3" t="n">
         <v>43132</v>
       </c>
       <c r="B39" t="n">
@@ -1878,7 +1879,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="3" t="n">
         <v>43160</v>
       </c>
       <c r="B40" t="n">
@@ -1892,7 +1893,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="3" t="n">
         <v>43191</v>
       </c>
       <c r="B41" t="n">
@@ -1906,7 +1907,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n">
+      <c r="A42" s="3" t="n">
         <v>43221</v>
       </c>
       <c r="B42" t="n">
@@ -1920,7 +1921,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="3" t="n">
         <v>43252</v>
       </c>
       <c r="B43" t="n">
@@ -1934,7 +1935,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n">
+      <c r="A44" s="3" t="n">
         <v>43282</v>
       </c>
       <c r="B44" t="n">
@@ -1948,7 +1949,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n">
+      <c r="A45" s="3" t="n">
         <v>43313</v>
       </c>
       <c r="B45" t="n">
@@ -1962,7 +1963,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="3" t="n">
         <v>43344</v>
       </c>
       <c r="B46" t="n">
@@ -1976,7 +1977,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="3" t="n">
         <v>43374</v>
       </c>
       <c r="B47" t="n">
@@ -1990,7 +1991,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="3" t="n">
         <v>43405</v>
       </c>
       <c r="B48" t="n">
@@ -2004,7 +2005,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n">
+      <c r="A49" s="3" t="n">
         <v>43435</v>
       </c>
       <c r="B49" t="n">
@@ -2018,7 +2019,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n">
+      <c r="A50" s="3" t="n">
         <v>43466</v>
       </c>
       <c r="B50" t="n">
@@ -2032,7 +2033,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n">
+      <c r="A51" s="3" t="n">
         <v>43497</v>
       </c>
       <c r="B51" t="n">
@@ -2046,7 +2047,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n">
+      <c r="A52" s="3" t="n">
         <v>43525</v>
       </c>
       <c r="B52" t="n">
@@ -2060,7 +2061,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="3" t="n">
         <v>43556</v>
       </c>
       <c r="B53" t="n">
@@ -2074,7 +2075,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="n">
+      <c r="A54" s="3" t="n">
         <v>43586</v>
       </c>
       <c r="B54" t="n">
@@ -2088,7 +2089,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="n">
+      <c r="A55" s="3" t="n">
         <v>43617</v>
       </c>
       <c r="B55" t="n">
@@ -2102,7 +2103,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="n">
+      <c r="A56" s="3" t="n">
         <v>43647</v>
       </c>
       <c r="B56" t="n">
@@ -2116,7 +2117,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="n">
+      <c r="A57" s="3" t="n">
         <v>43678</v>
       </c>
       <c r="B57" t="n">
@@ -2130,7 +2131,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="n">
+      <c r="A58" s="3" t="n">
         <v>43709</v>
       </c>
       <c r="B58" t="n">
@@ -2144,7 +2145,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="n">
+      <c r="A59" s="3" t="n">
         <v>43739</v>
       </c>
       <c r="B59" t="n">
@@ -2158,7 +2159,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="n">
+      <c r="A60" s="3" t="n">
         <v>43770</v>
       </c>
       <c r="B60" t="n">
@@ -2172,7 +2173,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="n">
+      <c r="A61" s="3" t="n">
         <v>43800</v>
       </c>
       <c r="B61" t="n">
@@ -2186,7 +2187,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="n">
+      <c r="A62" s="3" t="n">
         <v>43831</v>
       </c>
       <c r="B62" t="n">
@@ -2200,7 +2201,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="n">
+      <c r="A63" s="3" t="n">
         <v>43862</v>
       </c>
       <c r="B63" t="n">
@@ -2214,7 +2215,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="n">
+      <c r="A64" s="3" t="n">
         <v>43891</v>
       </c>
       <c r="B64" t="n">
@@ -2228,7 +2229,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="n">
+      <c r="A65" s="3" t="n">
         <v>43922</v>
       </c>
       <c r="B65" t="n">
@@ -2242,7 +2243,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="n">
+      <c r="A66" s="3" t="n">
         <v>43952</v>
       </c>
       <c r="B66" t="n">
@@ -2256,7 +2257,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="n">
+      <c r="A67" s="3" t="n">
         <v>43983</v>
       </c>
       <c r="B67" t="n">
@@ -2270,7 +2271,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="n">
+      <c r="A68" s="3" t="n">
         <v>44013</v>
       </c>
       <c r="B68" t="n">
@@ -2284,7 +2285,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="n">
+      <c r="A69" s="3" t="n">
         <v>44044</v>
       </c>
       <c r="B69" t="n">
@@ -2298,7 +2299,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="n">
+      <c r="A70" s="3" t="n">
         <v>44075</v>
       </c>
       <c r="B70" t="n">
@@ -2312,7 +2313,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="n">
+      <c r="A71" s="3" t="n">
         <v>44105</v>
       </c>
       <c r="B71" t="n">
@@ -2326,7 +2327,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="n">
+      <c r="A72" s="3" t="n">
         <v>44136</v>
       </c>
       <c r="B72" t="n">
@@ -2340,7 +2341,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="n">
+      <c r="A73" s="3" t="n">
         <v>44166</v>
       </c>
       <c r="B73" t="n">
@@ -2354,7 +2355,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="n">
+      <c r="A74" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B74" t="n">
@@ -2368,7 +2369,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="n">
+      <c r="A75" s="3" t="n">
         <v>44228</v>
       </c>
       <c r="B75" t="n">
@@ -2382,7 +2383,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="n">
+      <c r="A76" s="3" t="n">
         <v>44256</v>
       </c>
       <c r="B76" t="n">
@@ -2396,7 +2397,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="n">
+      <c r="A77" s="3" t="n">
         <v>44287</v>
       </c>
       <c r="B77" t="n">
@@ -2410,7 +2411,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="n">
+      <c r="A78" s="3" t="n">
         <v>44317</v>
       </c>
       <c r="B78" t="n">
@@ -2424,7 +2425,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="n">
+      <c r="A79" s="3" t="n">
         <v>44348</v>
       </c>
       <c r="B79" t="n">
@@ -2438,7 +2439,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="n">
+      <c r="A80" s="3" t="n">
         <v>44378</v>
       </c>
       <c r="B80" t="n">
@@ -2452,7 +2453,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="n">
+      <c r="A81" s="3" t="n">
         <v>44409</v>
       </c>
       <c r="B81" t="n">
@@ -2466,7 +2467,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="n">
+      <c r="A82" s="3" t="n">
         <v>44440</v>
       </c>
       <c r="B82" t="n">
@@ -2480,7 +2481,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="n">
+      <c r="A83" s="3" t="n">
         <v>44470</v>
       </c>
       <c r="B83" t="n">
@@ -2494,7 +2495,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="n">
+      <c r="A84" s="3" t="n">
         <v>44501</v>
       </c>
       <c r="B84" t="n">
@@ -2508,7 +2509,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="n">
+      <c r="A85" s="3" t="n">
         <v>44531</v>
       </c>
       <c r="B85" t="n">
@@ -2522,7 +2523,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="n">
+      <c r="A86" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B86" t="n">
@@ -2536,7 +2537,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="n">
+      <c r="A87" s="3" t="n">
         <v>44593</v>
       </c>
       <c r="B87" t="n">
@@ -2550,7 +2551,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="n">
+      <c r="A88" s="3" t="n">
         <v>44621</v>
       </c>
       <c r="B88" t="n">
@@ -2564,7 +2565,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="n">
+      <c r="A89" s="3" t="n">
         <v>44652</v>
       </c>
       <c r="B89" t="n">
@@ -2578,7 +2579,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="n">
+      <c r="A90" s="3" t="n">
         <v>44682</v>
       </c>
       <c r="B90" t="n">
@@ -2592,7 +2593,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="n">
+      <c r="A91" s="3" t="n">
         <v>44713</v>
       </c>
       <c r="B91" t="n">
@@ -2606,7 +2607,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="n">
+      <c r="A92" s="3" t="n">
         <v>44743</v>
       </c>
       <c r="B92" t="n">
@@ -2620,7 +2621,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="n">
+      <c r="A93" s="3" t="n">
         <v>44774</v>
       </c>
       <c r="B93" t="n">
@@ -2634,7 +2635,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="5" t="n">
+      <c r="A94" s="3" t="n">
         <v>44805</v>
       </c>
       <c r="B94" t="n">
@@ -2648,7 +2649,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="n">
+      <c r="A95" s="3" t="n">
         <v>44835</v>
       </c>
       <c r="B95" t="n">
@@ -2662,7 +2663,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="n">
+      <c r="A96" s="3" t="n">
         <v>44866</v>
       </c>
       <c r="B96" t="n">
@@ -2676,7 +2677,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="n">
+      <c r="A97" s="3" t="n">
         <v>44896</v>
       </c>
       <c r="B97" t="n">
@@ -2690,7 +2691,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="n">
+      <c r="A98" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B98" t="n">
@@ -2704,7 +2705,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="n">
+      <c r="A99" s="3" t="n">
         <v>44958</v>
       </c>
       <c r="B99" t="n">
@@ -2718,7 +2719,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="n">
+      <c r="A100" s="3" t="n">
         <v>44986</v>
       </c>
       <c r="B100" t="n">
@@ -2732,7 +2733,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="n">
+      <c r="A101" s="3" t="n">
         <v>45017</v>
       </c>
       <c r="B101" t="n">
@@ -2746,7 +2747,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="5" t="n">
+      <c r="A102" s="3" t="n">
         <v>45047</v>
       </c>
       <c r="B102" t="n">
@@ -2760,7 +2761,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="n">
+      <c r="A103" s="3" t="n">
         <v>45078</v>
       </c>
       <c r="B103" t="n">
@@ -2774,7 +2775,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="n">
+      <c r="A104" s="3" t="n">
         <v>45108</v>
       </c>
       <c r="B104" t="n">
@@ -2788,7 +2789,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="n">
+      <c r="A105" s="3" t="n">
         <v>45139</v>
       </c>
       <c r="B105" t="n">
@@ -2802,7 +2803,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="5" t="n">
+      <c r="A106" s="3" t="n">
         <v>45170</v>
       </c>
       <c r="B106" t="n">
@@ -2816,7 +2817,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="n">
+      <c r="A107" s="3" t="n">
         <v>45200</v>
       </c>
       <c r="B107" t="n">
@@ -2830,7 +2831,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="n">
+      <c r="A108" s="3" t="n">
         <v>45231</v>
       </c>
       <c r="B108" t="n">
@@ -2844,7 +2845,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="n">
+      <c r="A109" s="3" t="n">
         <v>45261</v>
       </c>
       <c r="B109" t="n">
@@ -2858,7 +2859,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="5" t="n">
+      <c r="A110" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B110" t="n">
@@ -2872,7 +2873,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="n">
+      <c r="A111" s="3" t="n">
         <v>45323</v>
       </c>
       <c r="B111" t="n">
@@ -2886,7 +2887,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="n">
+      <c r="A112" s="3" t="n">
         <v>45352</v>
       </c>
       <c r="B112" t="n">
@@ -2900,7 +2901,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="n">
+      <c r="A113" s="3" t="n">
         <v>45383</v>
       </c>
       <c r="B113" t="n">
@@ -2914,7 +2915,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="5" t="n">
+      <c r="A114" s="3" t="n">
         <v>45413</v>
       </c>
       <c r="B114" t="n">
@@ -2928,7 +2929,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="n">
+      <c r="A115" s="3" t="n">
         <v>45444</v>
       </c>
       <c r="B115" t="n">
@@ -2942,7 +2943,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="5" t="n">
+      <c r="A116" s="3" t="n">
         <v>45474</v>
       </c>
       <c r="B116" t="n">
@@ -2956,7 +2957,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="n">
+      <c r="A117" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="B117" t="n">
@@ -2970,7 +2971,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="5" t="n">
+      <c r="A118" s="3" t="n">
         <v>45536</v>
       </c>
       <c r="B118" t="n">
@@ -2984,7 +2985,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="n">
+      <c r="A119" s="3" t="n">
         <v>45566</v>
       </c>
       <c r="B119" t="n">
@@ -2998,7 +2999,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="5" t="n">
+      <c r="A120" s="3" t="n">
         <v>45597</v>
       </c>
       <c r="B120" t="n">
@@ -3012,7 +3013,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="n">
+      <c r="A121" s="3" t="n">
         <v>45627</v>
       </c>
       <c r="B121" t="n">
@@ -3026,7 +3027,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="n">
+      <c r="A122" s="3" t="n">
         <v>45658</v>
       </c>
       <c r="B122" t="n">
@@ -3040,7 +3041,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="n">
+      <c r="A123" s="3" t="n">
         <v>45689</v>
       </c>
       <c r="B123" t="n">
@@ -3054,7 +3055,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="5" t="n">
+      <c r="A124" s="3" t="n">
         <v>45717</v>
       </c>
       <c r="B124" t="n">
@@ -3068,7 +3069,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="n">
+      <c r="A125" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="B125" t="n">
@@ -3082,7 +3083,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="n">
+      <c r="A126" s="3" t="n">
         <v>45778</v>
       </c>
       <c r="B126" t="n">
@@ -3096,7 +3097,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="n">
+      <c r="A127" s="3" t="n">
         <v>45809</v>
       </c>
       <c r="B127" t="n">
@@ -3110,7 +3111,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="n">
+      <c r="A128" s="3" t="n">
         <v>45839</v>
       </c>
       <c r="B128" t="n">
@@ -3124,7 +3125,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="n">
+      <c r="A129" s="3" t="n">
         <v>45870</v>
       </c>
       <c r="B129" t="n">
@@ -3138,7 +3139,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="n">
+      <c r="A130" s="3" t="n">
         <v>45901</v>
       </c>
       <c r="B130" t="n">
@@ -3152,7 +3153,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="n">
+      <c r="A131" s="3" t="n">
         <v>45931</v>
       </c>
       <c r="B131" t="n">
@@ -3166,7 +3167,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="5" t="n">
+      <c r="A132" s="3" t="n">
         <v>45962</v>
       </c>
       <c r="B132" t="n">
@@ -3180,7 +3181,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="n">
+      <c r="A133" s="3" t="n">
         <v>45992</v>
       </c>
       <c r="B133" t="n">
@@ -3194,7 +3195,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="5" t="n">
+      <c r="A134" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="B134" t="n">
@@ -3208,7 +3209,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="n">
+      <c r="A135" s="3" t="n">
         <v>46054</v>
       </c>
       <c r="B135" t="n">
@@ -3222,7 +3223,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="n">
+      <c r="A136" s="3" t="n">
         <v>46082</v>
       </c>
       <c r="B136" t="n">
@@ -3236,7 +3237,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="n">
+      <c r="A137" s="3" t="n">
         <v>46113</v>
       </c>
       <c r="B137" t="n">
@@ -3250,7 +3251,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="5" t="n">
+      <c r="A138" s="3" t="n">
         <v>46143</v>
       </c>
       <c r="B138" t="n">
@@ -3264,7 +3265,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="n">
+      <c r="A139" s="3" t="n">
         <v>46174</v>
       </c>
       <c r="B139" t="n">
@@ -3278,7 +3279,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="5" t="n">
+      <c r="A140" s="3" t="n">
         <v>46204</v>
       </c>
       <c r="B140" t="n">
@@ -3352,7 +3353,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="3" t="n">
         <v>42005</v>
       </c>
       <c r="B2" t="n">
@@ -3375,7 +3376,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="3" t="n">
         <v>42036</v>
       </c>
       <c r="B3" t="n">
@@ -3398,7 +3399,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="3" t="n">
         <v>42064</v>
       </c>
       <c r="B4" t="n">
@@ -3421,7 +3422,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="3" t="n">
         <v>42095</v>
       </c>
       <c r="B5" t="n">
@@ -3444,7 +3445,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="3" t="n">
         <v>42125</v>
       </c>
       <c r="B6" t="n">
@@ -3467,7 +3468,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="3" t="n">
         <v>42156</v>
       </c>
       <c r="B7" t="n">
@@ -3490,7 +3491,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="3" t="n">
         <v>42186</v>
       </c>
       <c r="B8" t="n">
@@ -3513,7 +3514,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="3" t="n">
         <v>42217</v>
       </c>
       <c r="B9" t="n">
@@ -3536,7 +3537,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="3" t="n">
         <v>42248</v>
       </c>
       <c r="B10" t="n">
@@ -3559,7 +3560,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="3" t="n">
         <v>42278</v>
       </c>
       <c r="B11" t="n">
@@ -3582,7 +3583,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="3" t="n">
         <v>42309</v>
       </c>
       <c r="B12" t="n">
@@ -3605,7 +3606,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="3" t="n">
         <v>42339</v>
       </c>
       <c r="B13" t="n">
@@ -3628,7 +3629,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="3" t="n">
         <v>42370</v>
       </c>
       <c r="B14" t="n">
@@ -3651,7 +3652,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="3" t="n">
         <v>42401</v>
       </c>
       <c r="B15" t="n">
@@ -3674,7 +3675,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="3" t="n">
         <v>42430</v>
       </c>
       <c r="B16" t="n">
@@ -3697,7 +3698,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="3" t="n">
         <v>42461</v>
       </c>
       <c r="B17" t="n">
@@ -3720,7 +3721,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="3" t="n">
         <v>42491</v>
       </c>
       <c r="B18" t="n">
@@ -3743,7 +3744,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="3" t="n">
         <v>42522</v>
       </c>
       <c r="B19" t="n">
@@ -3766,7 +3767,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="3" t="n">
         <v>42552</v>
       </c>
       <c r="B20" t="n">
@@ -3792,7 +3793,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="3" t="n">
         <v>42583</v>
       </c>
       <c r="B21" t="n">
@@ -3818,7 +3819,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="3" t="n">
         <v>42614</v>
       </c>
       <c r="B22" t="n">
@@ -3844,7 +3845,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="3" t="n">
         <v>42644</v>
       </c>
       <c r="B23" t="n">
@@ -3870,7 +3871,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="3" t="n">
         <v>42675</v>
       </c>
       <c r="B24" t="n">
@@ -3896,7 +3897,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="3" t="n">
         <v>42705</v>
       </c>
       <c r="B25" t="n">
@@ -3922,7 +3923,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="3" t="n">
         <v>42736</v>
       </c>
       <c r="B26" t="n">
@@ -3948,7 +3949,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="3" t="n">
         <v>42767</v>
       </c>
       <c r="B27" t="n">
@@ -3974,7 +3975,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="3" t="n">
         <v>42795</v>
       </c>
       <c r="B28" t="n">
@@ -4000,7 +4001,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="3" t="n">
         <v>42826</v>
       </c>
       <c r="B29" t="n">
@@ -4026,7 +4027,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="3" t="n">
         <v>42856</v>
       </c>
       <c r="B30" t="n">
@@ -4052,7 +4053,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="3" t="n">
         <v>42887</v>
       </c>
       <c r="B31" t="n">
@@ -4078,7 +4079,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="3" t="n">
         <v>42917</v>
       </c>
       <c r="B32" t="n">
@@ -4104,7 +4105,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="3" t="n">
         <v>42948</v>
       </c>
       <c r="B33" t="n">
@@ -4130,7 +4131,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n">
+      <c r="A34" s="3" t="n">
         <v>42979</v>
       </c>
       <c r="B34" t="n">
@@ -4156,7 +4157,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="3" t="n">
         <v>43009</v>
       </c>
       <c r="B35" t="n">
@@ -4182,7 +4183,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="3" t="n">
         <v>43040</v>
       </c>
       <c r="B36" t="n">
@@ -4208,7 +4209,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="3" t="n">
         <v>43070</v>
       </c>
       <c r="B37" t="n">
@@ -4234,7 +4235,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n">
+      <c r="A38" s="3" t="n">
         <v>43101</v>
       </c>
       <c r="B38" t="n">
@@ -4260,7 +4261,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="3" t="n">
         <v>43132</v>
       </c>
       <c r="B39" t="n">
@@ -4286,7 +4287,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="3" t="n">
         <v>43160</v>
       </c>
       <c r="B40" t="n">
@@ -4312,7 +4313,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="3" t="n">
         <v>43191</v>
       </c>
       <c r="B41" t="n">
@@ -4338,7 +4339,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n">
+      <c r="A42" s="3" t="n">
         <v>43221</v>
       </c>
       <c r="B42" t="n">
@@ -4364,7 +4365,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="3" t="n">
         <v>43252</v>
       </c>
       <c r="B43" t="n">
@@ -4390,7 +4391,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n">
+      <c r="A44" s="3" t="n">
         <v>43282</v>
       </c>
       <c r="B44" t="n">
@@ -4416,7 +4417,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n">
+      <c r="A45" s="3" t="n">
         <v>43313</v>
       </c>
       <c r="B45" t="n">
@@ -4442,7 +4443,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="3" t="n">
         <v>43344</v>
       </c>
       <c r="B46" t="n">
@@ -4468,7 +4469,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="3" t="n">
         <v>43374</v>
       </c>
       <c r="B47" t="n">
@@ -4494,7 +4495,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="3" t="n">
         <v>43405</v>
       </c>
       <c r="B48" t="n">
@@ -4520,7 +4521,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n">
+      <c r="A49" s="3" t="n">
         <v>43435</v>
       </c>
       <c r="B49" t="n">
@@ -4546,7 +4547,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n">
+      <c r="A50" s="3" t="n">
         <v>43466</v>
       </c>
       <c r="B50" t="n">
@@ -4572,7 +4573,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n">
+      <c r="A51" s="3" t="n">
         <v>43497</v>
       </c>
       <c r="B51" t="n">
@@ -4598,7 +4599,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n">
+      <c r="A52" s="3" t="n">
         <v>43525</v>
       </c>
       <c r="B52" t="n">
@@ -4624,7 +4625,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="3" t="n">
         <v>43556</v>
       </c>
       <c r="B53" t="n">
@@ -4650,7 +4651,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="n">
+      <c r="A54" s="3" t="n">
         <v>43586</v>
       </c>
       <c r="B54" t="n">
@@ -4676,7 +4677,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="n">
+      <c r="A55" s="3" t="n">
         <v>43617</v>
       </c>
       <c r="B55" t="n">
@@ -4702,7 +4703,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="n">
+      <c r="A56" s="3" t="n">
         <v>43647</v>
       </c>
       <c r="B56" t="n">
@@ -4728,7 +4729,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="n">
+      <c r="A57" s="3" t="n">
         <v>43678</v>
       </c>
       <c r="B57" t="n">
@@ -4754,7 +4755,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="n">
+      <c r="A58" s="3" t="n">
         <v>43709</v>
       </c>
       <c r="B58" t="n">
@@ -4780,7 +4781,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="n">
+      <c r="A59" s="3" t="n">
         <v>43739</v>
       </c>
       <c r="B59" t="n">
@@ -4806,7 +4807,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="n">
+      <c r="A60" s="3" t="n">
         <v>43770</v>
       </c>
       <c r="B60" t="n">
@@ -4832,7 +4833,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="n">
+      <c r="A61" s="3" t="n">
         <v>43800</v>
       </c>
       <c r="B61" t="n">
@@ -4858,7 +4859,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="n">
+      <c r="A62" s="3" t="n">
         <v>43831</v>
       </c>
       <c r="B62" t="n">
@@ -4884,7 +4885,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="n">
+      <c r="A63" s="3" t="n">
         <v>43862</v>
       </c>
       <c r="B63" t="n">
@@ -4910,7 +4911,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="n">
+      <c r="A64" s="3" t="n">
         <v>43891</v>
       </c>
       <c r="B64" t="n">
@@ -4936,7 +4937,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="n">
+      <c r="A65" s="3" t="n">
         <v>43922</v>
       </c>
       <c r="B65" t="n">
@@ -4962,7 +4963,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="n">
+      <c r="A66" s="3" t="n">
         <v>43952</v>
       </c>
       <c r="B66" t="n">
@@ -4988,7 +4989,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="n">
+      <c r="A67" s="3" t="n">
         <v>43983</v>
       </c>
       <c r="B67" t="n">
@@ -5014,7 +5015,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="n">
+      <c r="A68" s="3" t="n">
         <v>44013</v>
       </c>
       <c r="B68" t="n">
@@ -5040,7 +5041,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="n">
+      <c r="A69" s="3" t="n">
         <v>44044</v>
       </c>
       <c r="B69" t="n">
@@ -5066,7 +5067,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="n">
+      <c r="A70" s="3" t="n">
         <v>44075</v>
       </c>
       <c r="B70" t="n">
@@ -5092,7 +5093,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="n">
+      <c r="A71" s="3" t="n">
         <v>44105</v>
       </c>
       <c r="B71" t="n">
@@ -5118,7 +5119,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="n">
+      <c r="A72" s="3" t="n">
         <v>44136</v>
       </c>
       <c r="B72" t="n">
@@ -5144,7 +5145,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="n">
+      <c r="A73" s="3" t="n">
         <v>44166</v>
       </c>
       <c r="B73" t="n">
@@ -5170,7 +5171,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="n">
+      <c r="A74" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B74" t="n">
@@ -5196,7 +5197,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="n">
+      <c r="A75" s="3" t="n">
         <v>44228</v>
       </c>
       <c r="B75" t="n">
@@ -5222,7 +5223,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="n">
+      <c r="A76" s="3" t="n">
         <v>44256</v>
       </c>
       <c r="B76" t="n">
@@ -5248,7 +5249,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="n">
+      <c r="A77" s="3" t="n">
         <v>44287</v>
       </c>
       <c r="B77" t="n">
@@ -5274,7 +5275,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="n">
+      <c r="A78" s="3" t="n">
         <v>44317</v>
       </c>
       <c r="B78" t="n">
@@ -5300,7 +5301,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="n">
+      <c r="A79" s="3" t="n">
         <v>44348</v>
       </c>
       <c r="B79" t="n">
@@ -5326,7 +5327,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="n">
+      <c r="A80" s="3" t="n">
         <v>44378</v>
       </c>
       <c r="B80" t="n">
@@ -5352,7 +5353,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="n">
+      <c r="A81" s="3" t="n">
         <v>44409</v>
       </c>
       <c r="B81" t="n">
@@ -5378,7 +5379,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="n">
+      <c r="A82" s="3" t="n">
         <v>44440</v>
       </c>
       <c r="B82" t="n">
@@ -5404,7 +5405,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="n">
+      <c r="A83" s="3" t="n">
         <v>44470</v>
       </c>
       <c r="B83" t="n">
@@ -5430,7 +5431,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="n">
+      <c r="A84" s="3" t="n">
         <v>44501</v>
       </c>
       <c r="B84" t="n">
@@ -5456,7 +5457,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="n">
+      <c r="A85" s="3" t="n">
         <v>44531</v>
       </c>
       <c r="B85" t="n">
@@ -5482,7 +5483,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="n">
+      <c r="A86" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B86" t="n">
@@ -5508,7 +5509,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="n">
+      <c r="A87" s="3" t="n">
         <v>44593</v>
       </c>
       <c r="B87" t="n">
@@ -5534,7 +5535,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="n">
+      <c r="A88" s="3" t="n">
         <v>44621</v>
       </c>
       <c r="B88" t="n">
@@ -5560,7 +5561,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="n">
+      <c r="A89" s="3" t="n">
         <v>44652</v>
       </c>
       <c r="B89" t="n">
@@ -5586,7 +5587,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="n">
+      <c r="A90" s="3" t="n">
         <v>44682</v>
       </c>
       <c r="B90" t="n">
@@ -5612,7 +5613,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="n">
+      <c r="A91" s="3" t="n">
         <v>44713</v>
       </c>
       <c r="B91" t="n">
@@ -5638,7 +5639,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="n">
+      <c r="A92" s="3" t="n">
         <v>44743</v>
       </c>
       <c r="B92" t="n">
@@ -5664,7 +5665,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="n">
+      <c r="A93" s="3" t="n">
         <v>44774</v>
       </c>
       <c r="B93" t="n">
@@ -5690,7 +5691,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="5" t="n">
+      <c r="A94" s="3" t="n">
         <v>44805</v>
       </c>
       <c r="B94" t="n">
@@ -5716,7 +5717,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="n">
+      <c r="A95" s="3" t="n">
         <v>44835</v>
       </c>
       <c r="B95" t="n">
@@ -5742,7 +5743,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="n">
+      <c r="A96" s="3" t="n">
         <v>44866</v>
       </c>
       <c r="B96" t="n">
@@ -5768,7 +5769,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="n">
+      <c r="A97" s="3" t="n">
         <v>44896</v>
       </c>
       <c r="B97" t="n">
@@ -5794,7 +5795,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="n">
+      <c r="A98" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B98" t="n">
@@ -5820,7 +5821,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="n">
+      <c r="A99" s="3" t="n">
         <v>44958</v>
       </c>
       <c r="B99" t="n">
@@ -5846,7 +5847,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="n">
+      <c r="A100" s="3" t="n">
         <v>44986</v>
       </c>
       <c r="B100" t="n">
@@ -5872,7 +5873,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="n">
+      <c r="A101" s="3" t="n">
         <v>45017</v>
       </c>
       <c r="B101" t="n">
@@ -5895,7 +5896,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="5" t="n">
+      <c r="A102" s="3" t="n">
         <v>45047</v>
       </c>
       <c r="B102" t="n">
@@ -5918,7 +5919,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="n">
+      <c r="A103" s="3" t="n">
         <v>45078</v>
       </c>
       <c r="B103" t="n">
@@ -5941,7 +5942,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="n">
+      <c r="A104" s="3" t="n">
         <v>45108</v>
       </c>
       <c r="B104" t="n">
@@ -5964,7 +5965,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="n">
+      <c r="A105" s="3" t="n">
         <v>45139</v>
       </c>
       <c r="B105" t="n">
@@ -5987,7 +5988,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="5" t="n">
+      <c r="A106" s="3" t="n">
         <v>45170</v>
       </c>
       <c r="B106" t="n">
@@ -6010,7 +6011,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="n">
+      <c r="A107" s="3" t="n">
         <v>45200</v>
       </c>
       <c r="B107" t="n">
@@ -6033,7 +6034,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="n">
+      <c r="A108" s="3" t="n">
         <v>45231</v>
       </c>
       <c r="B108" t="n">
@@ -6056,7 +6057,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="n">
+      <c r="A109" s="3" t="n">
         <v>45261</v>
       </c>
       <c r="B109" t="n">
@@ -6079,7 +6080,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="5" t="n">
+      <c r="A110" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B110" t="n">
@@ -6102,7 +6103,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="n">
+      <c r="A111" s="3" t="n">
         <v>45323</v>
       </c>
       <c r="B111" t="n">
@@ -6125,7 +6126,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="n">
+      <c r="A112" s="3" t="n">
         <v>45352</v>
       </c>
       <c r="B112" t="n">
@@ -6148,7 +6149,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="n">
+      <c r="A113" s="3" t="n">
         <v>45383</v>
       </c>
       <c r="B113" t="n">
@@ -6171,7 +6172,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="5" t="n">
+      <c r="A114" s="3" t="n">
         <v>45413</v>
       </c>
       <c r="B114" t="n">
@@ -6194,7 +6195,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="n">
+      <c r="A115" s="3" t="n">
         <v>45444</v>
       </c>
       <c r="B115" t="n">
@@ -6217,7 +6218,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="5" t="n">
+      <c r="A116" s="3" t="n">
         <v>45474</v>
       </c>
       <c r="B116" t="n">
@@ -6240,7 +6241,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="n">
+      <c r="A117" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="B117" t="n">
@@ -6263,7 +6264,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="5" t="n">
+      <c r="A118" s="3" t="n">
         <v>45536</v>
       </c>
       <c r="B118" t="n">
@@ -6286,7 +6287,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="n">
+      <c r="A119" s="3" t="n">
         <v>45566</v>
       </c>
       <c r="B119" t="n">
@@ -6309,7 +6310,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="5" t="n">
+      <c r="A120" s="3" t="n">
         <v>45597</v>
       </c>
       <c r="B120" t="n">
@@ -6332,7 +6333,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="n">
+      <c r="A121" s="3" t="n">
         <v>45627</v>
       </c>
       <c r="B121" t="n">
@@ -6355,7 +6356,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="n">
+      <c r="A122" s="3" t="n">
         <v>45658</v>
       </c>
       <c r="B122" t="n">
@@ -6378,7 +6379,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="n">
+      <c r="A123" s="3" t="n">
         <v>45689</v>
       </c>
       <c r="B123" t="n">
@@ -6401,7 +6402,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="5" t="n">
+      <c r="A124" s="3" t="n">
         <v>45717</v>
       </c>
       <c r="B124" t="n">
@@ -6424,7 +6425,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="n">
+      <c r="A125" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="B125" t="n">
@@ -6447,7 +6448,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="n">
+      <c r="A126" s="3" t="n">
         <v>45778</v>
       </c>
       <c r="B126" t="n">
@@ -6470,7 +6471,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="n">
+      <c r="A127" s="3" t="n">
         <v>45809</v>
       </c>
       <c r="B127" t="n">
@@ -6493,7 +6494,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="n">
+      <c r="A128" s="3" t="n">
         <v>45839</v>
       </c>
       <c r="B128" t="n">
@@ -6516,7 +6517,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="n">
+      <c r="A129" s="3" t="n">
         <v>45870</v>
       </c>
       <c r="B129" t="n">
@@ -6539,7 +6540,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="n">
+      <c r="A130" s="3" t="n">
         <v>45901</v>
       </c>
       <c r="B130" t="n">
@@ -6562,7 +6563,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="n">
+      <c r="A131" s="3" t="n">
         <v>45931</v>
       </c>
       <c r="B131" t="n">
@@ -6585,7 +6586,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="5" t="n">
+      <c r="A132" s="3" t="n">
         <v>45962</v>
       </c>
       <c r="B132" t="n">
@@ -6608,7 +6609,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="n">
+      <c r="A133" s="3" t="n">
         <v>45992</v>
       </c>
       <c r="B133" t="n">
@@ -6631,7 +6632,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="5" t="n">
+      <c r="A134" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="B134" t="n">
@@ -6654,7 +6655,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="n">
+      <c r="A135" s="3" t="n">
         <v>46054</v>
       </c>
       <c r="B135" t="n">
@@ -6677,7 +6678,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="n">
+      <c r="A136" s="3" t="n">
         <v>46082</v>
       </c>
       <c r="B136" t="n">
@@ -6700,7 +6701,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="n">
+      <c r="A137" s="3" t="n">
         <v>46113</v>
       </c>
       <c r="B137" t="n">
@@ -6723,7 +6724,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="5" t="n">
+      <c r="A138" s="3" t="n">
         <v>46143</v>
       </c>
       <c r="B138" t="n">
@@ -6746,7 +6747,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="n">
+      <c r="A139" s="3" t="n">
         <v>46174</v>
       </c>
       <c r="B139" t="n">
@@ -6769,7 +6770,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="5" t="n">
+      <c r="A140" s="3" t="n">
         <v>46204</v>
       </c>
       <c r="B140" t="n">
@@ -6837,7 +6838,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
+      <c r="A2" s="3" t="n">
         <v>42005</v>
       </c>
       <c r="B2" t="n">
@@ -6854,7 +6855,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="3" t="n">
         <v>42036</v>
       </c>
       <c r="B3" t="n">
@@ -6871,7 +6872,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="3" t="n">
         <v>42064</v>
       </c>
       <c r="B4" t="n">
@@ -6888,7 +6889,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="3" t="n">
         <v>42095</v>
       </c>
       <c r="B5" t="n">
@@ -6905,7 +6906,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="3" t="n">
         <v>42125</v>
       </c>
       <c r="B6" t="n">
@@ -6922,7 +6923,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="3" t="n">
         <v>42156</v>
       </c>
       <c r="B7" t="n">
@@ -6939,7 +6940,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="3" t="n">
         <v>42186</v>
       </c>
       <c r="B8" t="n">
@@ -6956,7 +6957,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="3" t="n">
         <v>42217</v>
       </c>
       <c r="B9" t="n">
@@ -6973,7 +6974,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="3" t="n">
         <v>42248</v>
       </c>
       <c r="B10" t="n">
@@ -6990,7 +6991,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="A11" s="3" t="n">
         <v>42278</v>
       </c>
       <c r="B11" t="n">
@@ -7007,7 +7008,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="3" t="n">
         <v>42309</v>
       </c>
       <c r="B12" t="n">
@@ -7024,7 +7025,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="3" t="n">
         <v>42339</v>
       </c>
       <c r="B13" t="n">
@@ -7041,7 +7042,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="3" t="n">
         <v>42370</v>
       </c>
       <c r="B14" t="n">
@@ -7058,7 +7059,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="3" t="n">
         <v>42401</v>
       </c>
       <c r="B15" t="n">
@@ -7075,7 +7076,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="3" t="n">
         <v>42430</v>
       </c>
       <c r="B16" t="n">
@@ -7092,7 +7093,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="A17" s="3" t="n">
         <v>42461</v>
       </c>
       <c r="B17" t="n">
@@ -7109,7 +7110,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="3" t="n">
         <v>42491</v>
       </c>
       <c r="B18" t="n">
@@ -7126,7 +7127,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="3" t="n">
         <v>42522</v>
       </c>
       <c r="B19" t="n">
@@ -7143,7 +7144,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="A20" s="3" t="n">
         <v>42552</v>
       </c>
       <c r="B20" t="n">
@@ -7160,7 +7161,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="3" t="n">
         <v>42583</v>
       </c>
       <c r="B21" t="n">
@@ -7177,7 +7178,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="3" t="n">
         <v>42614</v>
       </c>
       <c r="B22" t="n">
@@ -7194,7 +7195,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="A23" s="3" t="n">
         <v>42644</v>
       </c>
       <c r="B23" t="n">
@@ -7211,7 +7212,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="3" t="n">
         <v>42675</v>
       </c>
       <c r="B24" t="n">
@@ -7228,7 +7229,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="3" t="n">
         <v>42705</v>
       </c>
       <c r="B25" t="n">
@@ -7245,7 +7246,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="A26" s="3" t="n">
         <v>42736</v>
       </c>
       <c r="B26" t="n">
@@ -7262,7 +7263,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="3" t="n">
         <v>42767</v>
       </c>
       <c r="B27" t="n">
@@ -7279,7 +7280,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="3" t="n">
         <v>42795</v>
       </c>
       <c r="B28" t="n">
@@ -7296,7 +7297,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="A29" s="3" t="n">
         <v>42826</v>
       </c>
       <c r="B29" t="n">
@@ -7313,7 +7314,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="A30" s="3" t="n">
         <v>42856</v>
       </c>
       <c r="B30" t="n">
@@ -7330,7 +7331,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="A31" s="3" t="n">
         <v>42887</v>
       </c>
       <c r="B31" t="n">
@@ -7347,7 +7348,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="A32" s="3" t="n">
         <v>42917</v>
       </c>
       <c r="B32" t="n">
@@ -7364,7 +7365,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="A33" s="3" t="n">
         <v>42948</v>
       </c>
       <c r="B33" t="n">
@@ -7381,7 +7382,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="n">
+      <c r="A34" s="3" t="n">
         <v>42979</v>
       </c>
       <c r="B34" t="n">
@@ -7398,7 +7399,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="A35" s="3" t="n">
         <v>43009</v>
       </c>
       <c r="B35" t="n">
@@ -7415,7 +7416,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="A36" s="3" t="n">
         <v>43040</v>
       </c>
       <c r="B36" t="n">
@@ -7432,7 +7433,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="3" t="n">
         <v>43070</v>
       </c>
       <c r="B37" t="n">
@@ -7449,7 +7450,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="n">
+      <c r="A38" s="3" t="n">
         <v>43101</v>
       </c>
       <c r="B38" t="n">
@@ -7466,7 +7467,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="n">
+      <c r="A39" s="3" t="n">
         <v>43132</v>
       </c>
       <c r="B39" t="n">
@@ -7483,7 +7484,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="n">
+      <c r="A40" s="3" t="n">
         <v>43160</v>
       </c>
       <c r="B40" t="n">
@@ -7500,7 +7501,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="5" t="n">
+      <c r="A41" s="3" t="n">
         <v>43191</v>
       </c>
       <c r="B41" t="n">
@@ -7517,7 +7518,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="n">
+      <c r="A42" s="3" t="n">
         <v>43221</v>
       </c>
       <c r="B42" t="n">
@@ -7534,7 +7535,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="3" t="n">
         <v>43252</v>
       </c>
       <c r="B43" t="n">
@@ -7551,7 +7552,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="n">
+      <c r="A44" s="3" t="n">
         <v>43282</v>
       </c>
       <c r="B44" t="n">
@@ -7568,7 +7569,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="n">
+      <c r="A45" s="3" t="n">
         <v>43313</v>
       </c>
       <c r="B45" t="n">
@@ -7585,7 +7586,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="n">
+      <c r="A46" s="3" t="n">
         <v>43344</v>
       </c>
       <c r="B46" t="n">
@@ -7602,7 +7603,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n">
+      <c r="A47" s="3" t="n">
         <v>43374</v>
       </c>
       <c r="B47" t="n">
@@ -7619,7 +7620,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="3" t="n">
         <v>43405</v>
       </c>
       <c r="B48" t="n">
@@ -7636,7 +7637,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="n">
+      <c r="A49" s="3" t="n">
         <v>43435</v>
       </c>
       <c r="B49" t="n">
@@ -7653,7 +7654,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="n">
+      <c r="A50" s="3" t="n">
         <v>43466</v>
       </c>
       <c r="B50" t="n">
@@ -7670,7 +7671,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="n">
+      <c r="A51" s="3" t="n">
         <v>43497</v>
       </c>
       <c r="B51" t="n">
@@ -7687,7 +7688,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="n">
+      <c r="A52" s="3" t="n">
         <v>43525</v>
       </c>
       <c r="B52" t="n">
@@ -7704,7 +7705,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="5" t="n">
+      <c r="A53" s="3" t="n">
         <v>43556</v>
       </c>
       <c r="B53" t="n">
@@ -7721,7 +7722,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="5" t="n">
+      <c r="A54" s="3" t="n">
         <v>43586</v>
       </c>
       <c r="B54" t="n">
@@ -7738,7 +7739,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="5" t="n">
+      <c r="A55" s="3" t="n">
         <v>43617</v>
       </c>
       <c r="B55" t="n">
@@ -7755,7 +7756,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="n">
+      <c r="A56" s="3" t="n">
         <v>43647</v>
       </c>
       <c r="B56" t="n">
@@ -7772,7 +7773,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="n">
+      <c r="A57" s="3" t="n">
         <v>43678</v>
       </c>
       <c r="B57" t="n">
@@ -7789,7 +7790,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="n">
+      <c r="A58" s="3" t="n">
         <v>43709</v>
       </c>
       <c r="B58" t="n">
@@ -7806,7 +7807,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="n">
+      <c r="A59" s="3" t="n">
         <v>43739</v>
       </c>
       <c r="B59" t="n">
@@ -7823,7 +7824,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="n">
+      <c r="A60" s="3" t="n">
         <v>43770</v>
       </c>
       <c r="B60" t="n">
@@ -7840,7 +7841,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="n">
+      <c r="A61" s="3" t="n">
         <v>43800</v>
       </c>
       <c r="B61" t="n">
@@ -7857,7 +7858,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="n">
+      <c r="A62" s="3" t="n">
         <v>43831</v>
       </c>
       <c r="B62" t="n">
@@ -7874,7 +7875,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="n">
+      <c r="A63" s="3" t="n">
         <v>43862</v>
       </c>
       <c r="B63" t="n">
@@ -7891,7 +7892,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="5" t="n">
+      <c r="A64" s="3" t="n">
         <v>43891</v>
       </c>
       <c r="B64" t="n">
@@ -7908,7 +7909,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="n">
+      <c r="A65" s="3" t="n">
         <v>43922</v>
       </c>
       <c r="B65" t="n">
@@ -7925,7 +7926,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="5" t="n">
+      <c r="A66" s="3" t="n">
         <v>43952</v>
       </c>
       <c r="B66" t="n">
@@ -7942,7 +7943,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="n">
+      <c r="A67" s="3" t="n">
         <v>43983</v>
       </c>
       <c r="B67" t="n">
@@ -7959,7 +7960,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="n">
+      <c r="A68" s="3" t="n">
         <v>44013</v>
       </c>
       <c r="B68" t="n">
@@ -7976,7 +7977,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="n">
+      <c r="A69" s="3" t="n">
         <v>44044</v>
       </c>
       <c r="B69" t="n">
@@ -7993,7 +7994,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="n">
+      <c r="A70" s="3" t="n">
         <v>44075</v>
       </c>
       <c r="B70" t="n">
@@ -8010,7 +8011,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="n">
+      <c r="A71" s="3" t="n">
         <v>44105</v>
       </c>
       <c r="B71" t="n">
@@ -8027,7 +8028,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="n">
+      <c r="A72" s="3" t="n">
         <v>44136</v>
       </c>
       <c r="B72" t="n">
@@ -8044,7 +8045,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="n">
+      <c r="A73" s="3" t="n">
         <v>44166</v>
       </c>
       <c r="B73" t="n">
@@ -8061,7 +8062,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="n">
+      <c r="A74" s="3" t="n">
         <v>44197</v>
       </c>
       <c r="B74" t="n">
@@ -8078,7 +8079,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="5" t="n">
+      <c r="A75" s="3" t="n">
         <v>44228</v>
       </c>
       <c r="B75" t="n">
@@ -8095,7 +8096,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="5" t="n">
+      <c r="A76" s="3" t="n">
         <v>44256</v>
       </c>
       <c r="B76" t="n">
@@ -8112,7 +8113,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="5" t="n">
+      <c r="A77" s="3" t="n">
         <v>44287</v>
       </c>
       <c r="B77" t="n">
@@ -8129,7 +8130,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="n">
+      <c r="A78" s="3" t="n">
         <v>44317</v>
       </c>
       <c r="B78" t="n">
@@ -8146,7 +8147,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="n">
+      <c r="A79" s="3" t="n">
         <v>44348</v>
       </c>
       <c r="B79" t="n">
@@ -8163,7 +8164,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="n">
+      <c r="A80" s="3" t="n">
         <v>44378</v>
       </c>
       <c r="B80" t="n">
@@ -8180,7 +8181,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="n">
+      <c r="A81" s="3" t="n">
         <v>44409</v>
       </c>
       <c r="B81" t="n">
@@ -8197,7 +8198,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="n">
+      <c r="A82" s="3" t="n">
         <v>44440</v>
       </c>
       <c r="B82" t="n">
@@ -8214,7 +8215,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="n">
+      <c r="A83" s="3" t="n">
         <v>44470</v>
       </c>
       <c r="B83" t="n">
@@ -8231,7 +8232,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="n">
+      <c r="A84" s="3" t="n">
         <v>44501</v>
       </c>
       <c r="B84" t="n">
@@ -8248,7 +8249,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="n">
+      <c r="A85" s="3" t="n">
         <v>44531</v>
       </c>
       <c r="B85" t="n">
@@ -8265,7 +8266,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="n">
+      <c r="A86" s="3" t="n">
         <v>44562</v>
       </c>
       <c r="B86" t="n">
@@ -8282,7 +8283,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="5" t="n">
+      <c r="A87" s="3" t="n">
         <v>44593</v>
       </c>
       <c r="B87" t="n">
@@ -8299,7 +8300,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="5" t="n">
+      <c r="A88" s="3" t="n">
         <v>44621</v>
       </c>
       <c r="B88" t="n">
@@ -8316,7 +8317,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="5" t="n">
+      <c r="A89" s="3" t="n">
         <v>44652</v>
       </c>
       <c r="B89" t="n">
@@ -8333,7 +8334,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="5" t="n">
+      <c r="A90" s="3" t="n">
         <v>44682</v>
       </c>
       <c r="B90" t="n">
@@ -8350,7 +8351,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="5" t="n">
+      <c r="A91" s="3" t="n">
         <v>44713</v>
       </c>
       <c r="B91" t="n">
@@ -8367,7 +8368,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="5" t="n">
+      <c r="A92" s="3" t="n">
         <v>44743</v>
       </c>
       <c r="B92" t="n">
@@ -8384,7 +8385,7 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="5" t="n">
+      <c r="A93" s="3" t="n">
         <v>44774</v>
       </c>
       <c r="B93" t="n">
@@ -8401,7 +8402,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="5" t="n">
+      <c r="A94" s="3" t="n">
         <v>44805</v>
       </c>
       <c r="B94" t="n">
@@ -8418,7 +8419,7 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="5" t="n">
+      <c r="A95" s="3" t="n">
         <v>44835</v>
       </c>
       <c r="B95" t="n">
@@ -8435,7 +8436,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="5" t="n">
+      <c r="A96" s="3" t="n">
         <v>44866</v>
       </c>
       <c r="B96" t="n">
@@ -8452,7 +8453,7 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="5" t="n">
+      <c r="A97" s="3" t="n">
         <v>44896</v>
       </c>
       <c r="B97" t="n">
@@ -8469,7 +8470,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="n">
+      <c r="A98" s="3" t="n">
         <v>44927</v>
       </c>
       <c r="B98" t="n">
@@ -8486,7 +8487,7 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="n">
+      <c r="A99" s="3" t="n">
         <v>44958</v>
       </c>
       <c r="B99" t="n">
@@ -8503,7 +8504,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="5" t="n">
+      <c r="A100" s="3" t="n">
         <v>44986</v>
       </c>
       <c r="B100" t="n">
@@ -8520,7 +8521,7 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="5" t="n">
+      <c r="A101" s="3" t="n">
         <v>45017</v>
       </c>
       <c r="B101" t="n">
@@ -8537,7 +8538,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="5" t="n">
+      <c r="A102" s="3" t="n">
         <v>45047</v>
       </c>
       <c r="B102" t="n">
@@ -8554,7 +8555,7 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="5" t="n">
+      <c r="A103" s="3" t="n">
         <v>45078</v>
       </c>
       <c r="B103" t="n">
@@ -8571,7 +8572,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="5" t="n">
+      <c r="A104" s="3" t="n">
         <v>45108</v>
       </c>
       <c r="B104" t="n">
@@ -8588,7 +8589,7 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="5" t="n">
+      <c r="A105" s="3" t="n">
         <v>45139</v>
       </c>
       <c r="B105" t="n">
@@ -8605,7 +8606,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="5" t="n">
+      <c r="A106" s="3" t="n">
         <v>45170</v>
       </c>
       <c r="B106" t="n">
@@ -8622,7 +8623,7 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="5" t="n">
+      <c r="A107" s="3" t="n">
         <v>45200</v>
       </c>
       <c r="B107" t="n">
@@ -8639,7 +8640,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="n">
+      <c r="A108" s="3" t="n">
         <v>45231</v>
       </c>
       <c r="B108" t="n">
@@ -8656,7 +8657,7 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="5" t="n">
+      <c r="A109" s="3" t="n">
         <v>45261</v>
       </c>
       <c r="B109" t="n">
@@ -8673,7 +8674,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="5" t="n">
+      <c r="A110" s="3" t="n">
         <v>45292</v>
       </c>
       <c r="B110" t="n">
@@ -8690,7 +8691,7 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="5" t="n">
+      <c r="A111" s="3" t="n">
         <v>45323</v>
       </c>
       <c r="B111" t="n">
@@ -8707,7 +8708,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="n">
+      <c r="A112" s="3" t="n">
         <v>45352</v>
       </c>
       <c r="B112" t="n">
@@ -8724,7 +8725,7 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="5" t="n">
+      <c r="A113" s="3" t="n">
         <v>45383</v>
       </c>
       <c r="B113" t="n">
@@ -8741,7 +8742,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="5" t="n">
+      <c r="A114" s="3" t="n">
         <v>45413</v>
       </c>
       <c r="B114" t="n">
@@ -8758,7 +8759,7 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="5" t="n">
+      <c r="A115" s="3" t="n">
         <v>45444</v>
       </c>
       <c r="B115" t="n">
@@ -8775,7 +8776,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="5" t="n">
+      <c r="A116" s="3" t="n">
         <v>45474</v>
       </c>
       <c r="B116" t="n">
@@ -8792,7 +8793,7 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="5" t="n">
+      <c r="A117" s="3" t="n">
         <v>45505</v>
       </c>
       <c r="B117" t="n">
@@ -8809,7 +8810,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="5" t="n">
+      <c r="A118" s="3" t="n">
         <v>45536</v>
       </c>
       <c r="B118" t="n">
@@ -8826,7 +8827,7 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="5" t="n">
+      <c r="A119" s="3" t="n">
         <v>45566</v>
       </c>
       <c r="B119" t="n">
@@ -8843,7 +8844,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="5" t="n">
+      <c r="A120" s="3" t="n">
         <v>45597</v>
       </c>
       <c r="B120" t="n">
@@ -8860,7 +8861,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="5" t="n">
+      <c r="A121" s="3" t="n">
         <v>45627</v>
       </c>
       <c r="B121" t="n">
@@ -8877,7 +8878,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="5" t="n">
+      <c r="A122" s="3" t="n">
         <v>45658</v>
       </c>
       <c r="B122" t="n">
@@ -8894,7 +8895,7 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="5" t="n">
+      <c r="A123" s="3" t="n">
         <v>45689</v>
       </c>
       <c r="B123" t="n">
@@ -8911,7 +8912,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="5" t="n">
+      <c r="A124" s="3" t="n">
         <v>45717</v>
       </c>
       <c r="B124" t="n">
@@ -8928,7 +8929,7 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="5" t="n">
+      <c r="A125" s="3" t="n">
         <v>45748</v>
       </c>
       <c r="B125" t="n">
@@ -8945,7 +8946,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="5" t="n">
+      <c r="A126" s="3" t="n">
         <v>45778</v>
       </c>
       <c r="B126" t="n">
@@ -8962,7 +8963,7 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="5" t="n">
+      <c r="A127" s="3" t="n">
         <v>45809</v>
       </c>
       <c r="B127" t="n">
@@ -8979,7 +8980,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="5" t="n">
+      <c r="A128" s="3" t="n">
         <v>45839</v>
       </c>
       <c r="B128" t="n">
@@ -8996,7 +8997,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="5" t="n">
+      <c r="A129" s="3" t="n">
         <v>45870</v>
       </c>
       <c r="B129" t="n">
@@ -9013,7 +9014,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="5" t="n">
+      <c r="A130" s="3" t="n">
         <v>45901</v>
       </c>
       <c r="B130" t="n">
@@ -9030,7 +9031,7 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="5" t="n">
+      <c r="A131" s="3" t="n">
         <v>45931</v>
       </c>
       <c r="B131" t="n">
@@ -9047,7 +9048,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="5" t="n">
+      <c r="A132" s="3" t="n">
         <v>45962</v>
       </c>
       <c r="B132" t="n">
@@ -9064,7 +9065,7 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="n">
+      <c r="A133" s="3" t="n">
         <v>45992</v>
       </c>
       <c r="B133" t="n">
@@ -9081,7 +9082,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="5" t="n">
+      <c r="A134" s="3" t="n">
         <v>46023</v>
       </c>
       <c r="B134" t="n">
@@ -9098,7 +9099,7 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="n">
+      <c r="A135" s="3" t="n">
         <v>46054</v>
       </c>
       <c r="B135" t="n">
@@ -9115,7 +9116,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="5" t="n">
+      <c r="A136" s="3" t="n">
         <v>46082</v>
       </c>
       <c r="B136" t="n">
@@ -9132,7 +9133,7 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="5" t="n">
+      <c r="A137" s="3" t="n">
         <v>46113</v>
       </c>
       <c r="B137" t="n">
@@ -9149,7 +9150,7 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="5" t="n">
+      <c r="A138" s="3" t="n">
         <v>46143</v>
       </c>
       <c r="B138" t="n">
@@ -9166,7 +9167,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="5" t="n">
+      <c r="A139" s="3" t="n">
         <v>46174</v>
       </c>
       <c r="B139" t="n">
@@ -9183,7 +9184,7 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="5" t="n">
+      <c r="A140" s="3" t="n">
         <v>46204</v>
       </c>
       <c r="B140" t="n">

</xml_diff>